<commit_message>
Ora chiusura nel file del turno dopo, data della notte, cassaforte
- I24 (ORA CHIUSURA) è l'orario del terminale del turno precedente: quello inserito alla
  chiusura va nel file imbastito; il turno chiuso usa quello memorizzato dal turno prima
- la notte prende la data del giorno dopo (aperta alle 22 del 4 = notte del 5);
  successivo: pomeriggio del 4 -> notte del 5 -> mattina del 5
- popup "In cassaforte" alla chiusura: I28 nel turno chiuso e in quello dopo; i contanti
  attesi nel cassetto (D34) la escludono, l'avanzo del turno dopo la include
- prova_turno.sh: controlli su I24, I28 e stato salvato; esempi rigenerati

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FrvyfCDpgZPeDZbLuRno1S
</commit_message>
<xml_diff>
--- a/esempi/esempio_turno_chiuso.xlsx
+++ b/esempi/esempio_turno_chiuso.xlsx
@@ -1958,7 +1958,7 @@
       <c r="G20" s="88" t="n"/>
       <c r="H20" s="6" t="n"/>
       <c r="I20" s="84" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="J20" s="87" t="n"/>
       <c r="K20" s="88" t="n"/>
@@ -2098,9 +2098,7 @@
       <c r="F24" s="87" t="n"/>
       <c r="G24" s="88" t="n"/>
       <c r="H24" s="6" t="n"/>
-      <c r="I24" s="74" t="n">
-        <v>0.5871759259259259</v>
-      </c>
+      <c r="I24" s="74" t="n"/>
       <c r="J24" s="87" t="n"/>
       <c r="K24" s="88" t="n"/>
       <c r="L24" s="1" t="inlineStr">
@@ -2238,7 +2236,9 @@
       <c r="F28" s="87" t="n"/>
       <c r="G28" s="88" t="n"/>
       <c r="H28" s="6" t="n"/>
-      <c r="I28" s="45" t="n"/>
+      <c r="I28" s="45" t="n">
+        <v>20</v>
+      </c>
       <c r="J28" s="87" t="n"/>
       <c r="K28" s="88" t="n"/>
       <c r="L28" s="100" t="n"/>
@@ -2446,7 +2446,7 @@
       <c r="B34" s="87" t="n"/>
       <c r="C34" s="88" t="n"/>
       <c r="D34" s="6" t="n">
-        <v>150.5</v>
+        <v>130.5</v>
       </c>
       <c r="E34" s="55" t="inlineStr">
         <is>

</xml_diff>